<commit_message>
fix: supplier matching in PAKD import & contract form dropdown
</commit_message>
<xml_diff>
--- a/docs/templates/template_import_contracts.xlsx
+++ b/docs/templates/template_import_contracts.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Template" sheetId="1" r:id="rId1"/>
+    <sheet name="Import Hợp đồng" sheetId="1" r:id="rId1"/>
+    <sheet name="Hướng dẫn" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,139 +398,488 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:N4"/>
   <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="25.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+    <col min="1" max="1" width="5.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="18.83203125" customWidth="1"/>
+    <col min="14" max="14" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Tên hợp đồng</v>
+        <v>STT</v>
       </c>
       <c r="B1" t="str">
-        <v>Loại HĐ</v>
+        <v>Mã hợp đồng (*)</v>
       </c>
       <c r="C1" t="str">
-        <v>Khách hàng</v>
+        <v>Tên khách hàng (*)</v>
       </c>
       <c r="D1" t="str">
-        <v>Mã đơn vị</v>
+        <v>Đầu mối liên hệ</v>
       </c>
       <c r="E1" t="str">
-        <v>NVKD</v>
+        <v>Nội dung HĐ</v>
       </c>
       <c r="F1" t="str">
-        <v>Giá trị</v>
+        <v>Giá trị ký kết</v>
       </c>
       <c r="G1" t="str">
-        <v>Chi phí DK</v>
+        <v>Ngày ký (DD/MM/YYYY)</v>
       </c>
       <c r="H1" t="str">
-        <v>Ngày ký</v>
+        <v>Giá trị nghiệm thu</v>
       </c>
       <c r="I1" t="str">
-        <v>Ngày BĐ</v>
+        <v>Ngày nghiệm thu</v>
       </c>
       <c r="J1" t="str">
-        <v>Ngày KT</v>
+        <v>Doanh thu xuất HĐ</v>
       </c>
       <c r="K1" t="str">
-        <v>Trạng thái</v>
+        <v>Ngày xuất HĐ</v>
       </c>
       <c r="L1" t="str">
-        <v>Loại</v>
+        <v>Đã thanh toán</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Ngày thanh toán</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Còn lại</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>01.PPXD-CICHD2026</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Công ty TNHH ABC</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Nguyễn Văn A</v>
+      </c>
+      <c r="E2" t="str">
+        <v>BIM</v>
+      </c>
+      <c r="F2">
+        <v>500000000</v>
+      </c>
+      <c r="G2" t="str">
+        <v>15/01/2026</v>
+      </c>
+      <c r="H2">
+        <v>450000000</v>
+      </c>
+      <c r="I2" t="str">
+        <v>15/03/2026</v>
+      </c>
+      <c r="J2">
+        <v>450000000</v>
+      </c>
+      <c r="K2" t="str">
+        <v>20/03/2026</v>
+      </c>
+      <c r="L2">
+        <v>300000000</v>
+      </c>
+      <c r="M2" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="N2">
+        <v>150000000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>02.BIM-CICHD2026</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Tổng công ty XYZ</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Trần Thị B</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Tư vấn BIM</v>
+      </c>
+      <c r="F3">
+        <v>1200000000</v>
+      </c>
+      <c r="G3" t="str">
+        <v>20/02/2026</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>03.TVGS-CICHD2026</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Công ty CP DEF</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v>TVGS</v>
+      </c>
+      <c r="F4">
+        <v>800000000</v>
+      </c>
+      <c r="G4" t="str">
+        <v>01/03/2026</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:N4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D26"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="55.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>HƯỚNG DẪN IMPORT HỢP ĐỒNG - CIC ERP</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>HĐ Tư vấn dự án ABC</v>
-      </c>
-      <c r="B2" t="str">
-        <v>HĐ</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Công ty ABC</v>
-      </c>
-      <c r="D2" t="str">
-        <v>BIM</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Nguyễn Văn A</v>
-      </c>
-      <c r="F2">
-        <v>500000000</v>
-      </c>
-      <c r="G2">
-        <v>350000000</v>
-      </c>
-      <c r="H2" t="str">
-        <v>2024-01-15</v>
-      </c>
-      <c r="I2" t="str">
-        <v>2024-01-20</v>
-      </c>
-      <c r="J2" t="str">
-        <v>2024-06-30</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Active</v>
-      </c>
-      <c r="L2" t="str">
-        <v>Mới</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>HĐ Thiết kế XYZ</v>
+        <v>Cột</v>
       </c>
       <c r="B3" t="str">
-        <v>HĐNT</v>
+        <v>Mô tả</v>
       </c>
       <c r="C3" t="str">
-        <v>Tập đoàn XYZ</v>
+        <v>Bắt buộc</v>
       </c>
       <c r="D3" t="str">
-        <v>CSS</v>
-      </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-      <c r="F3">
-        <v>800000000</v>
-      </c>
-      <c r="G3">
-        <v>600000000</v>
-      </c>
-      <c r="H3" t="str">
-        <v>2024-02-01</v>
-      </c>
-      <c r="I3" t="str">
-        <v/>
-      </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
-      <c r="K3" t="str">
-        <v>Pending</v>
-      </c>
-      <c r="L3" t="str">
-        <v>Tiếp nối</v>
+        <v>Định dạng / Ghi chú</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>STT</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Số thứ tự</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Không</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Số tự nhiên (1, 2, 3...)</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Mã hợp đồng (*)</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Mã số hợp đồng duy nhất</v>
+      </c>
+      <c r="C5" t="str">
+        <v>CÓ</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Ví dụ: 01.PPXD-CICHD2026. Tránh ký tự / (sẽ tự chuyển thành -)</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Tên khách hàng (*)</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Tên công ty đối tác</v>
+      </c>
+      <c r="C6" t="str">
+        <v>CÓ</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Hệ thống sẽ tự tìm KH có sẵn hoặc tạo mới</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Đầu mối liên hệ</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Tên người liên hệ chính</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Không</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Sẽ lưu vào danh sách liên hệ của HĐ</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Nội dung HĐ</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Loại dịch vụ / phân loại</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Không</v>
+      </c>
+      <c r="D8" t="str">
+        <v>VD: BIM, Tư vấn BIM, TVGS, Thiết kế...</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Giá trị ký kết</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Giá trị hợp đồng đã ký</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Không</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Số nguyên, không dấu phân cách (VD: 500000000)</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Ngày ký</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Ngày ký hợp đồng</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Không</v>
+      </c>
+      <c r="D10" t="str">
+        <v>DD/MM/YYYY (VD: 15/01/2026)</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Giá trị nghiệm thu</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Tổng giá trị đã nghiệm thu</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Không</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Số nguyên</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Ngày nghiệm thu</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Ngày nghiệm thu gần nhất</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Không</v>
+      </c>
+      <c r="D12" t="str">
+        <v>DD/MM/YYYY</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Doanh thu xuất HĐ</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Tổng doanh thu đã xuất hóa đơn</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Không</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Số nguyên</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Ngày xuất HĐ</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Ngày xuất hóa đơn gần nhất</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Không</v>
+      </c>
+      <c r="D14" t="str">
+        <v>DD/MM/YYYY</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Đã thanh toán</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Tổng số tiền đã thu</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Không</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Số nguyên</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Ngày thanh toán</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Ngày thanh toán gần nhất</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Không</v>
+      </c>
+      <c r="D16" t="str">
+        <v>DD/MM/YYYY</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Còn lại</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Số tiền chưa thu</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Không</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Số nguyên (= Ký kết - Đã thanh toán)</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>LƯU Ý QUAN TRỌNG:</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>1. Các cột có dấu (*) là BẮT BUỘC phải có dữ liệu.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>2. Giá trị tiền tệ: nhập SỐ NGUYÊN, không dấu chấm/phẩy (VD: 500000000 chứ không phải 500.000.000).</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>3. Ngày tháng: DD/MM/YYYY.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>4. Mã HĐ đã tồn tại → CẬP NHẬT. Chưa có → TẠO MỚI.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>5. Khách hàng tìm theo tên. Không tìm thấy → tạo KH mới.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>6. Ký tự / trong Mã HĐ sẽ tự chuyển thành - khi tạo ID.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>7. XÓA dữ liệu mẫu trước khi import.</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D26"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>